<commit_message>
modified InvetoryFormPage with action methods, called those method in PurchaseOrderTest and added data into excel file
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/TestData.xlsx
+++ b/src/test/resources/TestData/TestData.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\ApplePurchaseOrder\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF3DAE9-1B83-4A91-A0CC-EAD66616FE83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58918888-2D5B-425D-A0E0-76936A6B19D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Credential" sheetId="1" r:id="rId1"/>
+    <sheet name="InventoryData" sheetId="2" r:id="rId2"/>
+    <sheet name="ExtraData" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Username</t>
   </si>
@@ -37,6 +39,51 @@
   </si>
   <si>
     <t>P@ssword</t>
+  </si>
+  <si>
+    <t>Device Type</t>
+  </si>
+  <si>
+    <t>Brand</t>
+  </si>
+  <si>
+    <t>Storage</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>123 Test Street</t>
+  </si>
+  <si>
+    <t>128GB</t>
+  </si>
+  <si>
+    <t>Shipping</t>
+  </si>
+  <si>
+    <t>Warranty</t>
+  </si>
+  <si>
+    <t>Express</t>
+  </si>
+  <si>
+    <t>1 Year</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>Blue</t>
   </si>
 </sst>
 </file>
@@ -395,4 +442,84 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9BEC3F2-D40B-4A83-BC99-C328B75A4793}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21ABB0BC-3D41-4793-81AD-57A519172A70}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
modified InvetoryFormPage with action methods, called those method in PurchaseOrderTest and added data into excel file again
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/TestData.xlsx
+++ b/src/test/resources/TestData/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\ApplePurchaseOrder\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58918888-2D5B-425D-A0E0-76936A6B19D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B21D08B-A658-49D8-BE05-3CBCFF0CC926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Credential" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Username</t>
   </si>
@@ -84,6 +84,18 @@
   </si>
   <si>
     <t>Blue</t>
+  </si>
+  <si>
+    <t>Discount</t>
+  </si>
+  <si>
+    <t>Save10</t>
+  </si>
+  <si>
+    <t>PurchaseMessage</t>
+  </si>
+  <si>
+    <t>Order Successful! 🎉</t>
   </si>
 </sst>
 </file>
@@ -500,26 +512,42 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21ABB0BC-3D41-4793-81AD-57A519172A70}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="4" max="4" width="34" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>12</v>
       </c>
       <c r="B1" t="s">
         <v>13</v>
       </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>14</v>
       </c>
       <c r="B2" t="s">
         <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>